<commit_message>
Clean generated artifacts from repository
</commit_message>
<xml_diff>
--- a/vulcan_mapping_with_atlas_reference_adj.xlsx
+++ b/vulcan_mapping_with_atlas_reference_adj.xlsx
@@ -1,32 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/raeltonhonorio/Documents/KDAM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{975A4F4E-C8A4-CA44-A34B-5FE7226BCD0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A1FA9D7-3602-1B40-B498-0162B2ED0620}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Vulcan Mapping" sheetId="1" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" r:id="rId2"/>
-    <sheet name="Atlas Official Names" sheetId="3" r:id="rId3"/>
-    <sheet name="VULCAN_OUTPUTS" sheetId="5" r:id="rId4"/>
-    <sheet name="VULCAN_MEDIA" sheetId="6" r:id="rId5"/>
-    <sheet name="VULCAN_SETUPS" sheetId="7" r:id="rId6"/>
-    <sheet name="Instructions" sheetId="4" r:id="rId7"/>
+    <sheet name="Sheet1" sheetId="8" r:id="rId2"/>
+    <sheet name="Summary" sheetId="2" r:id="rId3"/>
+    <sheet name="Atlas Official Names" sheetId="3" r:id="rId4"/>
+    <sheet name="VULCAN_OUTPUTS" sheetId="5" r:id="rId5"/>
+    <sheet name="VULCAN_MEDIA" sheetId="6" r:id="rId6"/>
+    <sheet name="VULCAN_SETUPS" sheetId="7" r:id="rId7"/>
+    <sheet name="Instructions" sheetId="4" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Atlas Official Names'!$A$2:$C$173</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Vulcan Mapping'!$A$1:$J$46</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">VULCAN_MEDIA!$A$1:$A$50</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">VULCAN_OUTPUTS!$A$1:$A$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">VULCAN_SETUPS!$A$1:$A$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Atlas Official Names'!$A$2:$C$173</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Vulcan Mapping'!$A$1:$K$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">VULCAN_MEDIA!$A$1:$A$50</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">VULCAN_OUTPUTS!$A$1:$A$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">VULCAN_SETUPS!$A$1:$A$73</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -46,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="961" uniqueCount="351">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="970" uniqueCount="361">
   <si>
     <t>VULCAN_SETUP</t>
   </si>
@@ -1099,13 +1100,43 @@
   </si>
   <si>
     <t>Ac no white under</t>
+  </si>
+  <si>
+    <t>Atlas MAX+ Color STD.icm</t>
+  </si>
+  <si>
+    <t>Avalanche</t>
+  </si>
+  <si>
+    <t>Atlas Max</t>
+  </si>
+  <si>
+    <t>Children pallet V3 (spring) Large</t>
+  </si>
+  <si>
+    <t>Children pallet V3 (spring) Small</t>
+  </si>
+  <si>
+    <t>Standard pallet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RSS - 15.9x19.9 </t>
+  </si>
+  <si>
+    <t>RSS - 11x15</t>
+  </si>
+  <si>
+    <t>RSS - 10.6x13.2</t>
+  </si>
+  <si>
+    <t>Fixa</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -1136,6 +1167,17 @@
       <b/>
       <sz val="16"/>
       <name val="Carlito"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Helvetica"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="major"/>
     </font>
   </fonts>
   <fills count="18">
@@ -1184,12 +1226,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF83E28E"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="3" tint="0.89999084444715716"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -1234,6 +1270,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFBE2D5"/>
         <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -1329,7 +1371,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1353,25 +1395,26 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -1384,6 +1427,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1586,1077 +1633,1173 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J46"/>
+  <dimension ref="A1:K46"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="25.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="33.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="35.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="29.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="29.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="36.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="24.1640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="20" customWidth="1"/>
+    <col min="2" max="2" width="25.6640625" customWidth="1"/>
+    <col min="3" max="3" width="33.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="7" width="29.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="29.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="36.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="24.1640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="16">
+    <row r="1" spans="1:11" ht="16">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="9" t="s">
+        <v>360</v>
+      </c>
+      <c r="C1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="D1" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="E1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="F1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="G1" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="H1" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="I1" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="J1" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="10" t="s">
+      <c r="K1" s="10" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:11" ht="16">
       <c r="A2" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="41"/>
+      <c r="C2" s="24" t="s">
         <v>348</v>
       </c>
-      <c r="C2" s="24" t="s">
+      <c r="D2" s="24" t="s">
         <v>346</v>
       </c>
-      <c r="D2" s="24" t="s">
+      <c r="E2" s="24" t="s">
         <v>329</v>
       </c>
-      <c r="E2" s="28" t="s">
+      <c r="F2" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="F2" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="G2" s="24" t="s">
-        <v>13</v>
-      </c>
-      <c r="H2" s="24" t="s">
-        <v>322</v>
-      </c>
-      <c r="I2" s="29" t="s">
+      <c r="G2" s="35" t="s">
+        <v>163</v>
+      </c>
+      <c r="H2" s="35" t="s">
+        <v>171</v>
+      </c>
+      <c r="I2" s="35" t="s">
+        <v>351</v>
+      </c>
+      <c r="J2" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="J2" s="14"/>
-    </row>
-    <row r="3" spans="1:10">
+      <c r="K2" s="14"/>
+    </row>
+    <row r="3" spans="1:11">
       <c r="A3" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="27" t="s">
+      <c r="B3" s="42"/>
+      <c r="C3" s="27" t="s">
         <v>347</v>
       </c>
-      <c r="C3" s="27" t="s">
+      <c r="D3" s="27" t="s">
         <v>346</v>
       </c>
-      <c r="D3" s="27" t="s">
+      <c r="E3" s="27" t="s">
         <v>335</v>
       </c>
-      <c r="E3" s="27" t="s">
+      <c r="F3" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="F3" s="23" t="s">
+      <c r="G3" s="23" t="s">
         <v>177</v>
       </c>
-      <c r="G3" s="27" t="s">
+      <c r="H3" s="27" t="s">
         <v>177</v>
       </c>
-      <c r="H3" s="27" t="s">
+      <c r="I3" s="27" t="s">
         <v>325</v>
       </c>
-      <c r="I3" s="29" t="s">
+      <c r="J3" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="J3" s="14"/>
-    </row>
-    <row r="4" spans="1:10">
+      <c r="K3" s="14"/>
+    </row>
+    <row r="4" spans="1:11" ht="16">
       <c r="A4" s="11"/>
-      <c r="C4" s="16" t="s">
+      <c r="B4" s="43"/>
+      <c r="D4" s="16" t="s">
         <v>346</v>
       </c>
-      <c r="D4" s="16" t="s">
+      <c r="E4" s="16" t="s">
         <v>331</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>18</v>
       </c>
-      <c r="F4" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="G4" s="24" t="s">
-        <v>13</v>
-      </c>
-      <c r="H4" s="24" t="s">
-        <v>322</v>
-      </c>
-      <c r="I4" s="29" t="s">
+      <c r="G4" s="35" t="s">
+        <v>163</v>
+      </c>
+      <c r="H4" s="35" t="s">
+        <v>171</v>
+      </c>
+      <c r="I4" s="35" t="s">
+        <v>351</v>
+      </c>
+      <c r="J4" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="J4" s="14"/>
-    </row>
-    <row r="5" spans="1:10">
+      <c r="K4" s="14"/>
+    </row>
+    <row r="5" spans="1:11" ht="16">
       <c r="A5" s="11"/>
-      <c r="C5" s="16" t="s">
+      <c r="B5" s="43"/>
+      <c r="D5" s="16" t="s">
         <v>346</v>
       </c>
-      <c r="D5" s="16" t="s">
+      <c r="E5" s="16" t="s">
         <v>332</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>18</v>
       </c>
-      <c r="F5" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="G5" s="24" t="s">
-        <v>13</v>
-      </c>
-      <c r="H5" s="24" t="s">
-        <v>322</v>
-      </c>
-      <c r="I5" s="29" t="s">
+      <c r="G5" s="35" t="s">
+        <v>163</v>
+      </c>
+      <c r="H5" s="35" t="s">
+        <v>171</v>
+      </c>
+      <c r="I5" s="35" t="s">
+        <v>351</v>
+      </c>
+      <c r="J5" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="J5" s="14"/>
-    </row>
-    <row r="6" spans="1:10">
+      <c r="K5" s="14"/>
+    </row>
+    <row r="6" spans="1:11" ht="16">
       <c r="A6" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="16"/>
+      <c r="C6" s="16" t="s">
         <v>349</v>
       </c>
-      <c r="C6" s="16" t="s">
+      <c r="D6" s="16" t="s">
         <v>346</v>
       </c>
-      <c r="D6" s="16" t="s">
+      <c r="E6" s="16" t="s">
         <v>329</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>18</v>
       </c>
-      <c r="F6" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6" s="24" t="s">
-        <v>13</v>
-      </c>
-      <c r="H6" s="30" t="s">
-        <v>322</v>
-      </c>
-      <c r="I6" s="29" t="s">
+      <c r="G6" s="35" t="s">
+        <v>163</v>
+      </c>
+      <c r="H6" s="35" t="s">
+        <v>171</v>
+      </c>
+      <c r="I6" s="35" t="s">
+        <v>351</v>
+      </c>
+      <c r="J6" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="J6" s="14"/>
-    </row>
-    <row r="7" spans="1:10">
+      <c r="K6" s="14"/>
+    </row>
+    <row r="7" spans="1:11" ht="16">
       <c r="A7" s="16" t="s">
         <v>123</v>
       </c>
       <c r="B7" s="16"/>
-      <c r="C7" s="16" t="s">
+      <c r="C7" s="16"/>
+      <c r="D7" s="16" t="s">
         <v>346</v>
       </c>
-      <c r="D7" s="16" t="s">
+      <c r="E7" s="16" t="s">
         <v>329</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>18</v>
       </c>
-      <c r="F7" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="G7" s="24" t="s">
-        <v>13</v>
-      </c>
-      <c r="H7" s="30" t="s">
-        <v>322</v>
-      </c>
-      <c r="I7" s="29" t="s">
+      <c r="G7" s="35" t="s">
+        <v>163</v>
+      </c>
+      <c r="H7" s="35" t="s">
+        <v>171</v>
+      </c>
+      <c r="I7" s="35" t="s">
+        <v>351</v>
+      </c>
+      <c r="J7" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="J7" s="14"/>
-    </row>
-    <row r="8" spans="1:10">
+      <c r="K7" s="14"/>
+    </row>
+    <row r="8" spans="1:11" ht="16">
       <c r="A8" s="16" t="s">
         <v>124</v>
       </c>
       <c r="B8" s="16"/>
-      <c r="C8" s="16" t="s">
+      <c r="C8" s="16"/>
+      <c r="D8" s="16" t="s">
         <v>346</v>
       </c>
-      <c r="D8" s="16" t="s">
+      <c r="E8" s="16" t="s">
         <v>329</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>18</v>
       </c>
-      <c r="F8" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="G8" s="24" t="s">
-        <v>13</v>
-      </c>
-      <c r="H8" s="30" t="s">
-        <v>322</v>
-      </c>
-      <c r="I8" s="29" t="s">
+      <c r="G8" s="35" t="s">
+        <v>163</v>
+      </c>
+      <c r="H8" s="35" t="s">
+        <v>171</v>
+      </c>
+      <c r="I8" s="35" t="s">
+        <v>351</v>
+      </c>
+      <c r="J8" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="J8" s="14"/>
-    </row>
-    <row r="9" spans="1:10">
+      <c r="K8" s="14"/>
+    </row>
+    <row r="9" spans="1:11" ht="16">
       <c r="A9" s="16" t="s">
         <v>125</v>
       </c>
       <c r="B9" s="16"/>
-      <c r="C9" s="16" t="s">
+      <c r="C9" s="16"/>
+      <c r="D9" s="16" t="s">
         <v>346</v>
       </c>
-      <c r="D9" s="16" t="s">
+      <c r="E9" s="16" t="s">
         <v>329</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F9" t="s">
         <v>18</v>
       </c>
-      <c r="F9" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="G9" s="24" t="s">
-        <v>13</v>
-      </c>
-      <c r="H9" s="30" t="s">
-        <v>322</v>
-      </c>
-      <c r="I9" s="29" t="s">
+      <c r="G9" s="35" t="s">
+        <v>163</v>
+      </c>
+      <c r="H9" s="35" t="s">
+        <v>171</v>
+      </c>
+      <c r="I9" s="35" t="s">
+        <v>351</v>
+      </c>
+      <c r="J9" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="J9" s="14"/>
-    </row>
-    <row r="10" spans="1:10">
+      <c r="K9" s="14"/>
+    </row>
+    <row r="10" spans="1:11" ht="16">
       <c r="A10" s="16" t="s">
         <v>126</v>
       </c>
       <c r="B10" s="16"/>
-      <c r="C10" s="16" t="s">
+      <c r="C10" s="16"/>
+      <c r="D10" s="16" t="s">
         <v>346</v>
       </c>
-      <c r="D10" s="16" t="s">
+      <c r="E10" s="16" t="s">
         <v>329</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
         <v>18</v>
       </c>
-      <c r="F10" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="G10" s="24" t="s">
-        <v>13</v>
-      </c>
-      <c r="H10" s="30" t="s">
-        <v>322</v>
-      </c>
-      <c r="I10" s="29" t="s">
+      <c r="G10" s="35" t="s">
+        <v>163</v>
+      </c>
+      <c r="H10" s="35" t="s">
+        <v>171</v>
+      </c>
+      <c r="I10" s="35" t="s">
+        <v>351</v>
+      </c>
+      <c r="J10" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="J10" s="14"/>
-    </row>
-    <row r="11" spans="1:10">
+      <c r="K10" s="14"/>
+    </row>
+    <row r="11" spans="1:11" ht="16">
       <c r="A11" s="16" t="s">
         <v>127</v>
       </c>
       <c r="B11" s="16"/>
-      <c r="C11" s="16" t="s">
+      <c r="C11" s="16"/>
+      <c r="D11" s="16" t="s">
         <v>346</v>
       </c>
-      <c r="D11" s="16" t="s">
+      <c r="E11" s="16" t="s">
         <v>329</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F11" t="s">
         <v>18</v>
       </c>
-      <c r="F11" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="G11" s="24" t="s">
-        <v>13</v>
-      </c>
-      <c r="H11" s="30" t="s">
-        <v>322</v>
-      </c>
-      <c r="I11" s="29" t="s">
+      <c r="G11" s="35" t="s">
+        <v>163</v>
+      </c>
+      <c r="H11" s="35" t="s">
+        <v>171</v>
+      </c>
+      <c r="I11" s="35" t="s">
+        <v>351</v>
+      </c>
+      <c r="J11" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="J11" s="14"/>
-    </row>
-    <row r="12" spans="1:10">
+      <c r="K11" s="14"/>
+    </row>
+    <row r="12" spans="1:11">
       <c r="A12" s="17" t="s">
         <v>100</v>
       </c>
-      <c r="B12" s="31"/>
-      <c r="C12" s="31" t="s">
+      <c r="B12" s="44"/>
+      <c r="C12" s="30"/>
+      <c r="D12" s="30" t="s">
         <v>346</v>
       </c>
-      <c r="D12" s="17" t="s">
+      <c r="E12" s="17" t="s">
         <v>334</v>
       </c>
-      <c r="E12" t="s">
+      <c r="F12" t="s">
         <v>18</v>
       </c>
-      <c r="F12" s="17" t="s">
+      <c r="G12" s="17" t="s">
         <v>175</v>
       </c>
-      <c r="G12" s="31" t="s">
+      <c r="H12" s="30" t="s">
         <v>175</v>
       </c>
-      <c r="H12" s="31" t="s">
+      <c r="I12" s="30" t="s">
         <v>324</v>
       </c>
-      <c r="I12" s="29" t="s">
+      <c r="J12" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="J12" s="14"/>
-    </row>
-    <row r="13" spans="1:10">
+      <c r="K12" s="14"/>
+    </row>
+    <row r="13" spans="1:11">
       <c r="A13" s="18" t="s">
         <v>102</v>
       </c>
       <c r="B13" s="18"/>
-      <c r="C13" s="18" t="s">
+      <c r="C13" s="18"/>
+      <c r="D13" s="18" t="s">
         <v>346</v>
       </c>
-      <c r="D13" s="18" t="s">
+      <c r="E13" s="18" t="s">
         <v>334</v>
       </c>
-      <c r="E13" t="s">
+      <c r="F13" t="s">
         <v>18</v>
       </c>
-      <c r="F13" s="18" t="s">
+      <c r="G13" s="18" t="s">
         <v>177</v>
       </c>
-      <c r="G13" s="32" t="s">
+      <c r="H13" s="31" t="s">
         <v>177</v>
       </c>
-      <c r="H13" s="32" t="s">
+      <c r="I13" s="31" t="s">
         <v>325</v>
       </c>
-      <c r="I13" s="29" t="s">
+      <c r="J13" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="J13" s="14"/>
-    </row>
-    <row r="14" spans="1:10">
+      <c r="K13" s="14"/>
+    </row>
+    <row r="14" spans="1:11">
       <c r="A14" s="25" t="s">
         <v>104</v>
       </c>
       <c r="B14" s="25"/>
-      <c r="C14" s="25" t="s">
+      <c r="C14" s="25"/>
+      <c r="D14" s="25" t="s">
         <v>346</v>
       </c>
-      <c r="D14" s="25" t="s">
+      <c r="E14" s="25" t="s">
         <v>334</v>
       </c>
-      <c r="E14" t="s">
+      <c r="F14" t="s">
         <v>18</v>
       </c>
-      <c r="F14" s="25" t="s">
+      <c r="G14" s="25" t="s">
         <v>90</v>
       </c>
-      <c r="G14" s="33" t="s">
+      <c r="H14" s="32" t="s">
         <v>90</v>
       </c>
-      <c r="H14" s="33" t="s">
+      <c r="I14" s="32" t="s">
         <v>323</v>
       </c>
-      <c r="I14" s="29" t="s">
+      <c r="J14" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="J14" s="14"/>
-    </row>
-    <row r="15" spans="1:10">
+      <c r="K14" s="14"/>
+    </row>
+    <row r="15" spans="1:11">
       <c r="A15" s="25" t="s">
         <v>106</v>
       </c>
       <c r="B15" s="25"/>
-      <c r="C15" s="25" t="s">
+      <c r="C15" s="25"/>
+      <c r="D15" s="25" t="s">
         <v>346</v>
       </c>
-      <c r="D15" s="25" t="s">
+      <c r="E15" s="25" t="s">
         <v>334</v>
       </c>
-      <c r="E15" t="s">
+      <c r="F15" t="s">
         <v>18</v>
       </c>
-      <c r="F15" s="19" t="s">
+      <c r="G15" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="G15" s="34" t="s">
+      <c r="H15" s="33" t="s">
         <v>90</v>
       </c>
-      <c r="H15" s="33" t="s">
+      <c r="I15" s="32" t="s">
         <v>323</v>
       </c>
-      <c r="I15" s="29" t="s">
+      <c r="J15" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="J15" s="14"/>
-    </row>
-    <row r="16" spans="1:10">
+      <c r="K15" s="14"/>
+    </row>
+    <row r="16" spans="1:11">
       <c r="A16" s="25" t="s">
         <v>108</v>
       </c>
       <c r="B16" s="25"/>
-      <c r="C16" s="25" t="s">
+      <c r="C16" s="25"/>
+      <c r="D16" s="25" t="s">
         <v>346</v>
       </c>
-      <c r="D16" s="25" t="s">
+      <c r="E16" s="25" t="s">
         <v>334</v>
       </c>
-      <c r="E16" t="s">
+      <c r="F16" t="s">
         <v>18</v>
       </c>
-      <c r="F16" s="19" t="s">
+      <c r="G16" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="G16" s="34" t="s">
+      <c r="H16" s="33" t="s">
         <v>90</v>
       </c>
-      <c r="H16" s="33" t="s">
+      <c r="I16" s="32" t="s">
         <v>323</v>
       </c>
-      <c r="I16" s="29" t="s">
+      <c r="J16" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="J16" s="14"/>
-    </row>
-    <row r="17" spans="1:10">
+      <c r="K16" s="14"/>
+    </row>
+    <row r="17" spans="1:11">
       <c r="A17" s="25" t="s">
         <v>110</v>
       </c>
       <c r="B17" s="25"/>
-      <c r="C17" s="25" t="s">
+      <c r="C17" s="25"/>
+      <c r="D17" s="25" t="s">
         <v>346</v>
       </c>
-      <c r="D17" s="25" t="s">
+      <c r="E17" s="25" t="s">
         <v>335</v>
       </c>
-      <c r="E17" t="s">
+      <c r="F17" t="s">
         <v>18</v>
       </c>
-      <c r="F17" s="25" t="s">
+      <c r="G17" s="25" t="s">
         <v>90</v>
       </c>
-      <c r="G17" s="33" t="s">
+      <c r="H17" s="32" t="s">
         <v>90</v>
       </c>
-      <c r="H17" s="33" t="s">
+      <c r="I17" s="32" t="s">
         <v>323</v>
       </c>
-      <c r="I17" s="29" t="s">
+      <c r="J17" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="J17" s="14"/>
-    </row>
-    <row r="18" spans="1:10">
+      <c r="K17" s="14"/>
+    </row>
+    <row r="18" spans="1:11">
       <c r="A18" s="17" t="s">
         <v>112</v>
       </c>
       <c r="B18" s="17"/>
-      <c r="C18" s="17" t="s">
+      <c r="C18" s="17"/>
+      <c r="D18" s="17" t="s">
         <v>346</v>
       </c>
-      <c r="D18" s="17" t="s">
+      <c r="E18" s="17" t="s">
         <v>334</v>
       </c>
-      <c r="E18" t="s">
+      <c r="F18" t="s">
         <v>18</v>
       </c>
-      <c r="F18" s="17" t="s">
+      <c r="G18" s="17" t="s">
         <v>175</v>
       </c>
-      <c r="G18" s="31" t="s">
+      <c r="H18" s="30" t="s">
         <v>175</v>
       </c>
-      <c r="H18" s="31" t="s">
+      <c r="I18" s="30" t="s">
         <v>324</v>
       </c>
-      <c r="I18" s="29" t="s">
+      <c r="J18" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="J18" s="14"/>
-    </row>
-    <row r="19" spans="1:10">
+      <c r="K18" s="14"/>
+    </row>
+    <row r="19" spans="1:11">
       <c r="A19" s="17" t="s">
         <v>114</v>
       </c>
       <c r="B19" s="17"/>
-      <c r="C19" s="17" t="s">
+      <c r="C19" s="17"/>
+      <c r="D19" s="17" t="s">
         <v>346</v>
       </c>
-      <c r="D19" s="17" t="s">
+      <c r="E19" s="17" t="s">
         <v>334</v>
       </c>
-      <c r="E19" t="s">
+      <c r="F19" t="s">
         <v>18</v>
       </c>
-      <c r="F19" s="17" t="s">
+      <c r="G19" s="17" t="s">
         <v>175</v>
       </c>
-      <c r="G19" s="31" t="s">
+      <c r="H19" s="30" t="s">
         <v>175</v>
       </c>
-      <c r="H19" s="31" t="s">
+      <c r="I19" s="30" t="s">
         <v>324</v>
       </c>
-      <c r="I19" s="29" t="s">
+      <c r="J19" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="J19" s="14"/>
-    </row>
-    <row r="20" spans="1:10">
+      <c r="K19" s="14"/>
+    </row>
+    <row r="20" spans="1:11">
       <c r="A20" s="17" t="s">
         <v>116</v>
       </c>
       <c r="B20" s="17"/>
-      <c r="C20" s="17" t="s">
+      <c r="C20" s="17"/>
+      <c r="D20" s="17" t="s">
         <v>346</v>
       </c>
-      <c r="D20" s="17" t="s">
+      <c r="E20" s="17" t="s">
         <v>335</v>
       </c>
-      <c r="E20" t="s">
+      <c r="F20" t="s">
         <v>18</v>
       </c>
-      <c r="F20" s="17" t="s">
+      <c r="G20" s="17" t="s">
         <v>175</v>
       </c>
-      <c r="G20" s="31" t="s">
+      <c r="H20" s="30" t="s">
         <v>175</v>
       </c>
-      <c r="H20" s="31" t="s">
+      <c r="I20" s="30" t="s">
         <v>324</v>
       </c>
-      <c r="I20" s="29" t="s">
+      <c r="J20" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="J20" s="14"/>
-    </row>
-    <row r="21" spans="1:10">
+      <c r="K20" s="14"/>
+    </row>
+    <row r="21" spans="1:11">
       <c r="A21" s="17" t="s">
         <v>118</v>
       </c>
       <c r="B21" s="17"/>
-      <c r="C21" s="17" t="s">
+      <c r="C21" s="17"/>
+      <c r="D21" s="17" t="s">
         <v>346</v>
       </c>
-      <c r="D21" s="17" t="s">
+      <c r="E21" s="17" t="s">
         <v>335</v>
       </c>
-      <c r="E21" t="s">
+      <c r="F21" t="s">
         <v>18</v>
       </c>
-      <c r="F21" s="17" t="s">
+      <c r="G21" s="17" t="s">
         <v>175</v>
       </c>
-      <c r="G21" s="31" t="s">
+      <c r="H21" s="30" t="s">
         <v>175</v>
       </c>
-      <c r="H21" s="31" t="s">
+      <c r="I21" s="30" t="s">
         <v>324</v>
       </c>
-      <c r="I21" s="29" t="s">
+      <c r="J21" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="J21" s="14"/>
-    </row>
-    <row r="22" spans="1:10">
+      <c r="K21" s="14"/>
+    </row>
+    <row r="22" spans="1:11">
       <c r="A22" s="17" t="s">
         <v>120</v>
       </c>
       <c r="B22" s="17"/>
-      <c r="C22" s="17" t="s">
+      <c r="C22" s="17"/>
+      <c r="D22" s="17" t="s">
         <v>346</v>
       </c>
-      <c r="D22" s="17" t="s">
+      <c r="E22" s="17" t="s">
         <v>335</v>
       </c>
-      <c r="E22" t="s">
+      <c r="F22" t="s">
         <v>18</v>
       </c>
-      <c r="F22" s="17" t="s">
+      <c r="G22" s="17" t="s">
         <v>175</v>
       </c>
-      <c r="G22" s="31" t="s">
+      <c r="H22" s="30" t="s">
         <v>175</v>
       </c>
-      <c r="H22" s="31" t="s">
+      <c r="I22" s="30" t="s">
         <v>324</v>
       </c>
-      <c r="I22" s="29" t="s">
+      <c r="J22" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="J22" s="14"/>
-    </row>
-    <row r="23" spans="1:10">
+      <c r="K22" s="14"/>
+    </row>
+    <row r="23" spans="1:11">
       <c r="A23" s="17" t="s">
         <v>122</v>
       </c>
       <c r="B23" s="17"/>
-      <c r="C23" s="17" t="s">
+      <c r="C23" s="17"/>
+      <c r="D23" s="17" t="s">
         <v>346</v>
       </c>
-      <c r="D23" s="17" t="s">
+      <c r="E23" s="17" t="s">
         <v>335</v>
       </c>
-      <c r="E23" t="s">
+      <c r="F23" t="s">
         <v>18</v>
       </c>
-      <c r="F23" s="17" t="s">
+      <c r="G23" s="17" t="s">
         <v>175</v>
       </c>
-      <c r="G23" s="31" t="s">
+      <c r="H23" s="30" t="s">
         <v>175</v>
       </c>
-      <c r="H23" s="31" t="s">
+      <c r="I23" s="30" t="s">
         <v>324</v>
       </c>
-      <c r="I23" s="29" t="s">
+      <c r="J23" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="J23" s="14"/>
-    </row>
-    <row r="24" spans="1:10">
+      <c r="K23" s="14"/>
+    </row>
+    <row r="24" spans="1:11">
       <c r="A24" s="18" t="s">
         <v>123</v>
       </c>
       <c r="B24" s="18"/>
-      <c r="C24" s="18" t="s">
+      <c r="C24" s="18"/>
+      <c r="D24" s="18" t="s">
         <v>346</v>
       </c>
-      <c r="D24" s="18" t="s">
+      <c r="E24" s="18" t="s">
         <v>334</v>
       </c>
-      <c r="E24" t="s">
+      <c r="F24" t="s">
         <v>18</v>
       </c>
-      <c r="F24" s="18" t="s">
+      <c r="G24" s="18" t="s">
         <v>177</v>
       </c>
-      <c r="G24" s="32" t="s">
+      <c r="H24" s="31" t="s">
         <v>177</v>
       </c>
-      <c r="H24" s="32" t="s">
+      <c r="I24" s="31" t="s">
         <v>325</v>
       </c>
-      <c r="I24" s="29" t="s">
+      <c r="J24" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="J24" s="14"/>
-    </row>
-    <row r="25" spans="1:10">
+      <c r="K24" s="14"/>
+    </row>
+    <row r="25" spans="1:11">
       <c r="A25" s="18" t="s">
         <v>124</v>
       </c>
       <c r="B25" s="18"/>
-      <c r="C25" s="18" t="s">
+      <c r="C25" s="18"/>
+      <c r="D25" s="18" t="s">
         <v>346</v>
       </c>
-      <c r="D25" s="18" t="s">
+      <c r="E25" s="18" t="s">
         <v>334</v>
       </c>
-      <c r="E25" t="s">
+      <c r="F25" t="s">
         <v>18</v>
       </c>
-      <c r="F25" s="26" t="s">
+      <c r="G25" s="26" t="s">
         <v>177</v>
       </c>
-      <c r="G25" s="35" t="s">
+      <c r="H25" s="34" t="s">
         <v>177</v>
       </c>
-      <c r="H25" s="35" t="s">
+      <c r="I25" s="34" t="s">
         <v>325</v>
       </c>
-      <c r="I25" s="29" t="s">
+      <c r="J25" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="J25" s="14"/>
-    </row>
-    <row r="26" spans="1:10">
+      <c r="K25" s="14"/>
+    </row>
+    <row r="26" spans="1:11">
       <c r="A26" s="18" t="s">
         <v>125</v>
       </c>
       <c r="B26" s="18"/>
-      <c r="C26" s="18" t="s">
+      <c r="C26" s="18"/>
+      <c r="D26" s="18" t="s">
         <v>346</v>
       </c>
-      <c r="D26" s="18" t="s">
+      <c r="E26" s="18" t="s">
         <v>335</v>
       </c>
-      <c r="E26" t="s">
+      <c r="F26" t="s">
         <v>18</v>
       </c>
-      <c r="F26" s="26" t="s">
+      <c r="G26" s="26" t="s">
         <v>177</v>
       </c>
-      <c r="G26" s="35" t="s">
+      <c r="H26" s="34" t="s">
         <v>177</v>
       </c>
-      <c r="H26" s="35" t="s">
+      <c r="I26" s="34" t="s">
         <v>325</v>
       </c>
-      <c r="I26" s="29" t="s">
+      <c r="J26" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="J26" s="14"/>
-    </row>
-    <row r="27" spans="1:10">
+      <c r="K26" s="14"/>
+    </row>
+    <row r="27" spans="1:11">
       <c r="A27" s="18" t="s">
         <v>126</v>
       </c>
       <c r="B27" s="18"/>
-      <c r="C27" s="18" t="s">
+      <c r="C27" s="18"/>
+      <c r="D27" s="18" t="s">
         <v>346</v>
       </c>
-      <c r="D27" s="18" t="s">
+      <c r="E27" s="18" t="s">
         <v>335</v>
       </c>
-      <c r="E27" t="s">
+      <c r="F27" t="s">
         <v>18</v>
       </c>
-      <c r="F27" s="26" t="s">
+      <c r="G27" s="26" t="s">
         <v>177</v>
       </c>
-      <c r="G27" s="35" t="s">
+      <c r="H27" s="34" t="s">
         <v>177</v>
       </c>
-      <c r="H27" s="35" t="s">
+      <c r="I27" s="34" t="s">
         <v>325</v>
       </c>
-      <c r="I27" s="29" t="s">
+      <c r="J27" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="J27" s="14"/>
-    </row>
-    <row r="28" spans="1:10">
+      <c r="K27" s="14"/>
+    </row>
+    <row r="28" spans="1:11">
       <c r="A28" s="18" t="s">
         <v>127</v>
       </c>
       <c r="B28" s="18"/>
-      <c r="C28" s="18" t="s">
+      <c r="C28" s="18"/>
+      <c r="D28" s="18" t="s">
         <v>346</v>
       </c>
-      <c r="D28" s="18" t="s">
+      <c r="E28" s="18" t="s">
         <v>335</v>
       </c>
-      <c r="E28" t="s">
+      <c r="F28" t="s">
         <v>18</v>
       </c>
-      <c r="F28" s="26" t="s">
+      <c r="G28" s="26" t="s">
         <v>177</v>
       </c>
-      <c r="G28" s="35" t="s">
+      <c r="H28" s="34" t="s">
         <v>177</v>
       </c>
-      <c r="H28" s="35" t="s">
+      <c r="I28" s="34" t="s">
         <v>325</v>
       </c>
-      <c r="I28" s="29" t="s">
+      <c r="J28" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="J28" s="14"/>
-    </row>
-    <row r="29" spans="1:10">
+      <c r="K28" s="14"/>
+    </row>
+    <row r="29" spans="1:11">
       <c r="A29" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="F29" s="11"/>
-      <c r="I29" s="29"/>
-      <c r="J29" s="14"/>
-    </row>
-    <row r="30" spans="1:10">
+      <c r="B29" s="43"/>
+      <c r="G29" s="11"/>
+      <c r="J29" s="29"/>
+      <c r="K29" s="14"/>
+    </row>
+    <row r="30" spans="1:11">
       <c r="A30" s="11" t="s">
         <v>129</v>
       </c>
-      <c r="F30" s="11"/>
-      <c r="I30" s="29"/>
-      <c r="J30" s="14"/>
-    </row>
-    <row r="31" spans="1:10">
+      <c r="B30" s="43"/>
+      <c r="G30" s="11"/>
+      <c r="J30" s="29"/>
+      <c r="K30" s="14"/>
+    </row>
+    <row r="31" spans="1:11">
       <c r="A31" s="11" t="s">
         <v>130</v>
       </c>
-      <c r="F31" s="11"/>
-      <c r="I31" s="29"/>
-      <c r="J31" s="14"/>
-    </row>
-    <row r="32" spans="1:10">
+      <c r="B31" s="43"/>
+      <c r="G31" s="11"/>
+      <c r="J31" s="29"/>
+      <c r="K31" s="14"/>
+    </row>
+    <row r="32" spans="1:11" ht="16">
       <c r="A32" s="16" t="s">
         <v>131</v>
       </c>
       <c r="B32" s="16"/>
-      <c r="C32" s="16" t="s">
+      <c r="C32" s="16"/>
+      <c r="D32" s="16" t="s">
         <v>346</v>
       </c>
-      <c r="D32" s="16" t="s">
+      <c r="E32" s="16" t="s">
         <v>329</v>
       </c>
-      <c r="E32" t="s">
+      <c r="F32" t="s">
         <v>18</v>
       </c>
-      <c r="F32" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="G32" s="24" t="s">
-        <v>13</v>
-      </c>
-      <c r="H32" s="30" t="s">
-        <v>322</v>
-      </c>
-      <c r="I32" s="29" t="s">
+      <c r="G32" s="35" t="s">
+        <v>163</v>
+      </c>
+      <c r="H32" s="35" t="s">
+        <v>171</v>
+      </c>
+      <c r="I32" s="35" t="s">
+        <v>351</v>
+      </c>
+      <c r="J32" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="J32" s="14"/>
-    </row>
-    <row r="33" spans="1:10">
+      <c r="K32" s="14"/>
+    </row>
+    <row r="33" spans="1:11" ht="16">
       <c r="A33" s="16" t="s">
         <v>132</v>
       </c>
       <c r="B33" s="16"/>
-      <c r="C33" s="16" t="s">
+      <c r="C33" s="16"/>
+      <c r="D33" s="16" t="s">
         <v>346</v>
       </c>
-      <c r="D33" s="16" t="s">
+      <c r="E33" s="16" t="s">
         <v>329</v>
       </c>
-      <c r="E33" t="s">
+      <c r="F33" t="s">
         <v>18</v>
       </c>
-      <c r="F33" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="G33" s="24" t="s">
-        <v>13</v>
-      </c>
-      <c r="H33" s="30" t="s">
-        <v>322</v>
-      </c>
-      <c r="I33" s="29" t="s">
+      <c r="G33" s="35" t="s">
+        <v>163</v>
+      </c>
+      <c r="H33" s="35" t="s">
+        <v>171</v>
+      </c>
+      <c r="I33" s="35" t="s">
+        <v>351</v>
+      </c>
+      <c r="J33" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="J33" s="14"/>
-    </row>
-    <row r="34" spans="1:10">
+      <c r="K33" s="14"/>
+    </row>
+    <row r="34" spans="1:11">
       <c r="A34" s="11" t="s">
         <v>133</v>
       </c>
-      <c r="C34" t="s">
+      <c r="B34" s="43"/>
+      <c r="D34" t="s">
         <v>346</v>
       </c>
-      <c r="D34" t="s">
+      <c r="E34" t="s">
         <v>335</v>
       </c>
-      <c r="E34" t="s">
+      <c r="F34" t="s">
         <v>18</v>
       </c>
-      <c r="F34" s="26" t="s">
+      <c r="G34" s="26" t="s">
         <v>177</v>
       </c>
-      <c r="G34" s="35" t="s">
+      <c r="H34" s="34" t="s">
         <v>177</v>
       </c>
-      <c r="H34" s="35" t="s">
+      <c r="I34" s="34" t="s">
         <v>325</v>
       </c>
-      <c r="I34" s="29" t="s">
+      <c r="J34" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="J34" s="14"/>
-    </row>
-    <row r="35" spans="1:10">
+      <c r="K34" s="14"/>
+    </row>
+    <row r="35" spans="1:11">
       <c r="A35" s="11" t="s">
         <v>134</v>
       </c>
-      <c r="E35" t="s">
+      <c r="B35" s="43"/>
+      <c r="F35" t="s">
         <v>12</v>
       </c>
-      <c r="F35" s="11"/>
-      <c r="J35" s="14"/>
-    </row>
-    <row r="36" spans="1:10">
+      <c r="G35" s="11"/>
+      <c r="K35" s="14"/>
+    </row>
+    <row r="36" spans="1:11">
       <c r="A36" s="11" t="s">
         <v>135</v>
       </c>
-      <c r="E36" t="s">
+      <c r="B36" s="43"/>
+      <c r="F36" t="s">
         <v>29</v>
       </c>
-      <c r="F36" s="11"/>
-      <c r="J36" s="14"/>
-    </row>
-    <row r="37" spans="1:10">
+      <c r="G36" s="11"/>
+      <c r="K36" s="14"/>
+    </row>
+    <row r="37" spans="1:11">
       <c r="A37" s="11" t="s">
         <v>136</v>
       </c>
-      <c r="E37" t="s">
+      <c r="B37" s="43"/>
+      <c r="F37" t="s">
         <v>12</v>
       </c>
-      <c r="F37" s="11"/>
-      <c r="J37" s="14"/>
-    </row>
-    <row r="38" spans="1:10">
+      <c r="G37" s="11"/>
+      <c r="K37" s="14"/>
+    </row>
+    <row r="38" spans="1:11">
       <c r="A38" s="11" t="s">
         <v>137</v>
       </c>
-      <c r="E38" t="s">
+      <c r="B38" s="43"/>
+      <c r="F38" t="s">
         <v>12</v>
       </c>
-      <c r="F38" s="11"/>
-      <c r="J38" s="14"/>
-    </row>
-    <row r="39" spans="1:10">
+      <c r="G38" s="11"/>
+      <c r="K38" s="14"/>
+    </row>
+    <row r="39" spans="1:11">
       <c r="A39" s="11" t="s">
         <v>138</v>
       </c>
-      <c r="E39" t="s">
+      <c r="B39" s="43"/>
+      <c r="F39" t="s">
         <v>12</v>
       </c>
-      <c r="F39" s="11"/>
-      <c r="J39" s="14"/>
-    </row>
-    <row r="40" spans="1:10">
+      <c r="G39" s="11"/>
+      <c r="K39" s="14"/>
+    </row>
+    <row r="40" spans="1:11">
       <c r="A40" s="11" t="s">
         <v>139</v>
       </c>
-      <c r="E40" t="s">
+      <c r="B40" s="43"/>
+      <c r="F40" t="s">
         <v>12</v>
       </c>
-      <c r="F40" s="11"/>
-      <c r="J40" s="14"/>
-    </row>
-    <row r="41" spans="1:10">
+      <c r="G40" s="11"/>
+      <c r="K40" s="14"/>
+    </row>
+    <row r="41" spans="1:11">
       <c r="A41" s="11" t="s">
         <v>140</v>
       </c>
-      <c r="E41" t="s">
+      <c r="B41" s="43"/>
+      <c r="F41" t="s">
         <v>12</v>
       </c>
-      <c r="F41" s="11"/>
-      <c r="J41" s="14"/>
-    </row>
-    <row r="42" spans="1:10">
+      <c r="G41" s="11"/>
+      <c r="K41" s="14"/>
+    </row>
+    <row r="42" spans="1:11">
       <c r="A42" s="11" t="s">
         <v>141</v>
       </c>
-      <c r="E42" t="s">
+      <c r="B42" s="43"/>
+      <c r="F42" t="s">
         <v>12</v>
       </c>
-      <c r="F42" s="11"/>
-      <c r="J42" s="14"/>
-    </row>
-    <row r="43" spans="1:10">
+      <c r="G42" s="11"/>
+      <c r="K42" s="14"/>
+    </row>
+    <row r="43" spans="1:11">
       <c r="A43" s="11" t="s">
         <v>142</v>
       </c>
-      <c r="E43" t="s">
+      <c r="B43" s="43"/>
+      <c r="F43" t="s">
         <v>12</v>
       </c>
-      <c r="F43" s="11"/>
-      <c r="J43" s="14"/>
-    </row>
-    <row r="44" spans="1:10">
+      <c r="G43" s="11"/>
+      <c r="K43" s="14"/>
+    </row>
+    <row r="44" spans="1:11">
       <c r="A44" s="11" t="s">
         <v>143</v>
       </c>
-      <c r="E44" t="s">
+      <c r="B44" s="43"/>
+      <c r="F44" t="s">
         <v>12</v>
       </c>
-      <c r="F44" s="11"/>
-      <c r="J44" s="14"/>
-    </row>
-    <row r="45" spans="1:10">
+      <c r="G44" s="11"/>
+      <c r="K44" s="14"/>
+    </row>
+    <row r="45" spans="1:11">
       <c r="A45" s="11" t="s">
         <v>350</v>
       </c>
-      <c r="C45" t="s">
+      <c r="B45" s="43"/>
+      <c r="D45" t="s">
         <v>346</v>
       </c>
-      <c r="D45" t="s">
+      <c r="E45" t="s">
         <v>335</v>
       </c>
-      <c r="E45" t="s">
+      <c r="F45" t="s">
         <v>18</v>
       </c>
-      <c r="F45" s="26" t="s">
+      <c r="G45" s="26" t="s">
         <v>177</v>
       </c>
-      <c r="G45" s="35" t="s">
+      <c r="H45" s="34" t="s">
         <v>177</v>
       </c>
-      <c r="H45" s="35" t="s">
+      <c r="I45" s="34" t="s">
         <v>325</v>
       </c>
-      <c r="I45" s="29" t="s">
+      <c r="J45" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="J45" s="14"/>
-    </row>
-    <row r="46" spans="1:10" ht="15" thickBot="1">
+      <c r="K45" s="14"/>
+    </row>
+    <row r="46" spans="1:11" ht="15" thickBot="1">
       <c r="A46" s="12" t="s">
         <v>144</v>
       </c>
       <c r="B46" s="13"/>
       <c r="C46" s="13"/>
       <c r="D46" s="13"/>
-      <c r="E46" s="13" t="s">
+      <c r="E46" s="13"/>
+      <c r="F46" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="F46" s="12"/>
-      <c r="G46" s="13"/>
+      <c r="G46" s="12"/>
       <c r="H46" s="13"/>
       <c r="I46" s="13"/>
-      <c r="J46" s="15"/>
+      <c r="J46" s="13"/>
+      <c r="K46" s="15"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J46" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
-  <conditionalFormatting sqref="E2:E46">
+  <autoFilter ref="A1:K46" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <conditionalFormatting sqref="F2:F46">
     <cfRule type="expression" dxfId="2" priority="1">
-      <formula>E2="mapped"</formula>
+      <formula>F2="mapped"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="1" priority="2">
-      <formula>E2="fallback"</formula>
+      <formula>F2="fallback"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="0" priority="3">
-      <formula>E2="review"</formula>
+      <formula>F2="review"</formula>
     </cfRule>
   </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29356F2C-C1AC-604E-9729-A12F153D775D}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14"/>
+  <cols>
+    <col min="1" max="1" width="30.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.1640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>352</v>
+      </c>
+      <c r="B1" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="15">
+      <c r="A2" t="s">
+        <v>354</v>
+      </c>
+      <c r="B2" s="36" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="15">
+      <c r="A3" t="s">
+        <v>355</v>
+      </c>
+      <c r="B3" s="36" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="15">
+      <c r="A4" t="s">
+        <v>356</v>
+      </c>
+      <c r="B4" s="36" t="s">
+        <v>357</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
@@ -2717,7 +2860,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr filterMode="1"/>
   <dimension ref="A1:C173"/>
@@ -2729,11 +2872,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="15">
-      <c r="A1" s="36" t="s">
+      <c r="A1" s="37" t="s">
         <v>153</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
     </row>
     <row r="2" spans="1:3" ht="15">
       <c r="A2" s="2" t="s">
@@ -4642,7 +4785,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3CEEBD3-5CC0-D048-93C2-13208FC84A91}">
   <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14"/>
@@ -4716,7 +4859,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FEA240F-6FD4-7540-AFF6-B358CDD85203}">
   <dimension ref="A1:A50"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14"/>
@@ -4980,7 +5123,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2858F9B9-1CE3-AD45-9AB8-712ADDBA836B}">
   <dimension ref="A1:A73"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14"/>
@@ -5359,7 +5502,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
@@ -5369,10 +5512,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="15">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="39" t="s">
         <v>305</v>
       </c>
-      <c r="B1" s="39"/>
+      <c r="B1" s="40"/>
     </row>
     <row r="2" spans="1:2" ht="15">
       <c r="A2" s="4" t="s">

</xml_diff>